<commit_message>
Fix AHR allele inputs and verify Sheets writes with global duplicate checks
</commit_message>
<xml_diff>
--- a/caffeine-sensitivity-app/assets/caffeine-atlas-batch-template.xlsx
+++ b/caffeine-sensitivity-app/assets/caffeine-atlas-batch-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="일괄 입력" sheetId="1" r:id="Rc19ac5fe432e41d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="2" r:id="Ra6ff490acebb48a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입력값 코드북" sheetId="3" r:id="Re346f4fe6f094f68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="일괄 입력" sheetId="1" r:id="R122f6f1290cb4e5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="2" r:id="Rdb237562eab44b66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입력값 코드북" sheetId="3" r:id="R21fca693baea4f3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -839,7 +839,7 @@
         <x:v>CC</x:v>
       </x:c>
       <x:c r="I2" s="27" t="str">
-        <x:v>GG</x:v>
+        <x:v>AA</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="18" customHeight="1">
@@ -3169,7 +3169,7 @@
         <x:v>SAMPLE-001</x:v>
       </x:c>
       <x:c r="E6" s="72" t="str">
-        <x:v>파일 안에서 중복 불가</x:v>
+        <x:v>파일·기존 시트 중복 불가</x:v>
       </x:c>
       <x:c r="F6" s="73" t="str">
         <x:v>이름·주민번호 대신 비식별 ID 권장</x:v>
@@ -3326,7 +3326,7 @@
         <x:v>목록 선택</x:v>
       </x:c>
       <x:c r="D14" s="78" t="str">
-        <x:v>GG / TG / TT / 모름</x:v>
+        <x:v>AA / AT / TT / 모름</x:v>
       </x:c>
       <x:c r="E14" s="78" t="str">
         <x:v>허용 유전자형</x:v>
@@ -3414,7 +3414,7 @@
         <x:v>CC</x:v>
       </x:c>
       <x:c r="F2" s="98" t="str">
-        <x:v>GG</x:v>
+        <x:v>AA</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3434,7 +3434,7 @@
         <x:v>CT</x:v>
       </x:c>
       <x:c r="F3" s="101" t="str">
-        <x:v>TG</x:v>
+        <x:v>AT</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>